<commit_message>
Add reservation-confirmation block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 10
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-confirmed.report.xlsx
+++ b/tools/importer/reports/import-jsw-confirmed.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="47">
   <si>
     <t>_reportFile</t>
   </si>
@@ -31,6 +31,9 @@
     <t>sections</t>
   </si>
   <si>
+    <t>split</t>
+  </si>
+  <si>
     <t>status</t>
   </si>
   <si>
@@ -82,13 +85,25 @@
     <t>MG Latest Luxury &amp; Electric Cars in India - Prices &amp; Models</t>
   </si>
   <si>
+    <t>jsw-confirmed-split.report.json</t>
+  </si>
+  <si>
+    <t>jsw-confirmed-split</t>
+  </si>
+  <si>
+    <t>2026-10-21T09:04:39.707Z</t>
+  </si>
+  <si>
+    <t>jsw-confirmed</t>
+  </si>
+  <si>
+    <t>https://example.com/?layout=split</t>
+  </si>
+  <si>
     <t>jsw-confirmed.report.json</t>
   </si>
   <si>
-    <t>jsw-confirmed</t>
-  </si>
-  <si>
-    <t>2026-10-21T07:34:48.619Z</t>
+    <t>2026-10-21T09:04:34.437Z</t>
   </si>
   <si>
     <t>https://example.com/</t>
@@ -525,22 +540,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="50" customWidth="1"/>
-    <col min="11" max="11" width="29" customWidth="1"/>
+    <col min="7" max="7" width="7" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="26" customWidth="1"/>
+    <col min="11" max="11" width="50" customWidth="1"/>
+    <col min="12" max="12" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -574,66 +590,72 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2">
         <v>4</v>
       </c>
       <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
         <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
       </c>
       <c r="I3" t="s">
         <v>21</v>
@@ -642,221 +664,280 @@
         <v>22</v>
       </c>
       <c r="K3" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I4" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K4" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="L4" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5">
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6">
         <v>9</v>
       </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" t="s">
-        <v>28</v>
-      </c>
-      <c r="K5" t="s">
-        <v>26</v>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L7" t="s">
         <v>31</v>
       </c>
-      <c r="F6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J6" t="s">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" t="s">
         <v>31</v>
       </c>
-      <c r="K6" t="s">
-        <v>26</v>
-      </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" t="s">
-        <v>35</v>
-      </c>
-      <c r="J7" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" t="s">
-        <v>26</v>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" t="s">
+        <v>43</v>
+      </c>
+      <c r="K9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L9" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" t="s">
-        <v>37</v>
-      </c>
-      <c r="K8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10">
         <v>5</v>
       </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" t="s">
-        <v>41</v>
-      </c>
-      <c r="J9" t="s">
-        <v>40</v>
-      </c>
-      <c r="K9" t="s">
-        <v>16</v>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" t="s">
+        <v>46</v>
+      </c>
+      <c r="K10" t="s">
+        <v>45</v>
+      </c>
+      <c r="L10" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add reservation-confirmation, reservation-form blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 16
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-confirmed.report.xlsx
+++ b/tools/importer/reports/import-jsw-confirmed.report.xlsx
@@ -91,7 +91,7 @@
     <t>jsw-confirmed-split</t>
   </si>
   <si>
-    <t>2026-10-21T09:04:39.707Z</t>
+    <t>2026-10-21T10:00:20.508Z</t>
   </si>
   <si>
     <t>jsw-confirmed</t>
@@ -103,7 +103,7 @@
     <t>jsw-confirmed.report.json</t>
   </si>
   <si>
-    <t>2026-10-21T09:04:34.437Z</t>
+    <t>2026-10-21T10:00:16.280Z</t>
   </si>
   <si>
     <t>https://example.com/</t>
@@ -133,7 +133,7 @@
     <t>jsw-reserve</t>
   </si>
   <si>
-    <t>2026-10-21T07:34:40.950Z</t>
+    <t>2026-10-21T10:00:08.954Z</t>
   </si>
   <si>
     <t>jsw-sustainability.report.json</t>

</xml_diff>

<commit_message>
Add reservation-form block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 16
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-confirmed.report.xlsx
+++ b/tools/importer/reports/import-jsw-confirmed.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="52">
   <si>
     <t>_reportFile</t>
   </si>
@@ -22,6 +22,9 @@
     <t>cards</t>
   </si>
   <si>
+    <t>failed</t>
+  </si>
+  <si>
     <t>images</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>jsw-confirmed-split</t>
   </si>
   <si>
-    <t>2026-10-21T10:44:14.786Z</t>
+    <t>2026-10-23T10:13:35.090Z</t>
   </si>
   <si>
     <t>jsw-confirmed</t>
@@ -103,7 +106,7 @@
     <t>jsw-confirmed.report.json</t>
   </si>
   <si>
-    <t>2026-10-21T10:44:09.971Z</t>
+    <t>2026-10-23T10:13:30.287Z</t>
   </si>
   <si>
     <t>https://example.com/</t>
@@ -118,6 +121,18 @@
     <t>2026-10-09T10:52:29.321Z</t>
   </si>
   <si>
+    <t>jsw-payment-failed.report.json</t>
+  </si>
+  <si>
+    <t>jsw-payment-failed</t>
+  </si>
+  <si>
+    <t>2026-10-23T10:13:40.519Z</t>
+  </si>
+  <si>
+    <t>https://example.com/?page=failed</t>
+  </si>
+  <si>
     <t>jsw-phase-3.report.json</t>
   </si>
   <si>
@@ -133,7 +148,7 @@
     <t>jsw-reserve</t>
   </si>
   <si>
-    <t>2026-10-21T10:44:03.061Z</t>
+    <t>2026-10-23T10:13:22.520Z</t>
   </si>
   <si>
     <t>jsw-sustainability.report.json</t>
@@ -540,23 +555,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="26" customWidth="1"/>
-    <col min="11" max="11" width="50" customWidth="1"/>
-    <col min="12" max="12" width="35" customWidth="1"/>
+    <col min="4" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="7" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="50" customWidth="1"/>
+    <col min="13" max="13" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,72 +608,78 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2">
         <v>4</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
         <v>16</v>
-      </c>
-      <c r="K2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>21</v>
       </c>
       <c r="J3" t="s">
         <v>22</v>
@@ -667,39 +688,42 @@
         <v>23</v>
       </c>
       <c r="L3" t="s">
-        <v>17</v>
+        <v>24</v>
+      </c>
+      <c r="M3" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="b">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="s">
-        <v>15</v>
-      </c>
       <c r="I4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="K4" t="s">
         <v>27</v>
@@ -707,237 +731,299 @@
       <c r="L4" t="s">
         <v>28</v>
       </c>
+      <c r="M4" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="b">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="b">
         <v>0</v>
       </c>
-      <c r="H5" t="s">
-        <v>15</v>
-      </c>
       <c r="I5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J5" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="K5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L5" t="s">
-        <v>31</v>
+        <v>28</v>
+      </c>
+      <c r="M5" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K6" t="s">
-        <v>33</v>
-      </c>
-      <c r="L6" t="s">
-        <v>31</v>
-      </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J7" t="s">
-        <v>37</v>
-      </c>
-      <c r="K7" t="s">
-        <v>36</v>
-      </c>
-      <c r="L7" t="s">
-        <v>31</v>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" t="s">
+        <v>42</v>
+      </c>
+      <c r="L8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M8" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" t="s">
-        <v>13</v>
-      </c>
-      <c r="J8" t="s">
-        <v>40</v>
-      </c>
-      <c r="K8" t="s">
-        <v>39</v>
-      </c>
-      <c r="L8" t="s">
-        <v>31</v>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" t="s">
+        <v>45</v>
+      </c>
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+      <c r="M9" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10">
         <v>6</v>
       </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" t="s">
-        <v>43</v>
-      </c>
-      <c r="K9" t="s">
-        <v>42</v>
-      </c>
-      <c r="L9" t="s">
-        <v>31</v>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" t="s">
+        <v>47</v>
+      </c>
+      <c r="M10" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11">
         <v>5</v>
       </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" t="s">
-        <v>46</v>
-      </c>
-      <c r="K10" t="s">
-        <v>45</v>
-      </c>
-      <c r="L10" t="s">
-        <v>17</v>
+      <c r="H11" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M11" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>